<commit_message>
chore(data): batch update intraday faturamento_realizado - 13:32:04
</commit_message>
<xml_diff>
--- a/data/faturamento_realizado.xlsx
+++ b/data/faturamento_realizado.xlsx
@@ -6195,7 +6195,7 @@
         <v>326</v>
       </c>
       <c r="D360" t="n">
-        <v>42942.24</v>
+        <v>43580.66</v>
       </c>
     </row>
     <row r="361">
@@ -10547,7 +10547,7 @@
         <v>42</v>
       </c>
       <c r="D632" t="n">
-        <v>435426.76</v>
+        <v>436132.48</v>
       </c>
     </row>
     <row r="633">
@@ -12755,7 +12755,7 @@
         <v>341</v>
       </c>
       <c r="D770" t="n">
-        <v>6252.69</v>
+        <v>6886.19</v>
       </c>
     </row>
     <row r="771">
@@ -12851,7 +12851,7 @@
         <v>1465</v>
       </c>
       <c r="D776" t="n">
-        <v>155103.66</v>
+        <v>156209.03</v>
       </c>
     </row>
     <row r="777">
@@ -15123,7 +15123,7 @@
         <v>1810</v>
       </c>
       <c r="D918" t="n">
-        <v>13596.67</v>
+        <v>16782.77</v>
       </c>
     </row>
     <row r="919">
@@ -17651,7 +17651,7 @@
         <v>40</v>
       </c>
       <c r="D1076" t="n">
-        <v>106317.23</v>
+        <v>106759.96</v>
       </c>
     </row>
     <row r="1077">

</xml_diff>